<commit_message>
#123 J1 Connector Update in PCB and fresh Deliverables Added
</commit_message>
<xml_diff>
--- a/Design-Files/ArmBand-Sensor-Board/BOM/Client BOM of ArmBand-Sensor-Board.xlsx
+++ b/Design-Files/ArmBand-Sensor-Board/BOM/Client BOM of ArmBand-Sensor-Board.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ManarHarake-sEMGDevice\Design-Files\ArmBand-Sensor-Board\Project Outputs for ArmBand-Sensor-Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ManarHarake-sEMGDevice\Design-Files\ArmBand-Sensor-Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C6DF28-6FFA-4A33-8C72-17C4A9F19719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -100,9 +99,6 @@
     <t>CAP CER 0.1UF 50V X7R 0402</t>
   </si>
   <si>
-    <t>Slide Lock 32P Contact,Top Surface Mount，Right Angle 0.5mm SMD,P=0.5mm,Surface Mount，Right Angle FFC/FPC Connectors ROHS</t>
-  </si>
-  <si>
     <t>CONN FPC/FFC 12POS .5MM</t>
   </si>
   <si>
@@ -139,9 +135,6 @@
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>AFC07-S32ECA-00</t>
-  </si>
-  <si>
     <t>FH34SRJ-12S-0.5SH(50)_</t>
   </si>
   <si>
@@ -251,12 +244,18 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>AFC07-S32FCA-00</t>
+  </si>
+  <si>
+    <t>Slide Lock 32P Bottom Contact Surface Mount 0.5mm SMD,P=0.5mm FFC/FPC Connectors ROHS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -836,7 +835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -879,19 +878,19 @@
         <v>23</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -908,16 +907,16 @@
         <v>24</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J3" s="15">
         <v>3</v>
@@ -939,22 +938,22 @@
         <v>25</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J4" s="17">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="21">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -967,19 +966,19 @@
         <v>12</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>39</v>
+        <v>75</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>75</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>75</v>
       </c>
       <c r="J5" s="15">
         <v>1</v>
@@ -998,19 +997,19 @@
         <v>13</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J6" s="17">
         <v>1</v>
@@ -1027,19 +1026,19 @@
         <v>14</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F7" s="15" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J7" s="15">
         <v>11</v>
@@ -1058,16 +1057,16 @@
         <v>15</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I8" s="18" t="s">
         <v>5</v>
@@ -1087,19 +1086,19 @@
         <v>16</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J9" s="15">
         <v>2</v>
@@ -1118,19 +1117,19 @@
         <v>17</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J10" s="17">
         <v>2</v>
@@ -1147,19 +1146,19 @@
         <v>18</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J11" s="15">
         <v>6</v>
@@ -1178,19 +1177,19 @@
         <v>19</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I12" s="18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J12" s="17">
         <v>2</v>
@@ -1209,19 +1208,19 @@
         <v>20</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J13" s="15">
         <v>1</v>
@@ -1240,19 +1239,19 @@
         <v>21</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J14" s="17">
         <v>1</v>
@@ -1269,19 +1268,19 @@
         <v>22</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J15" s="15">
         <v>2</v>

</xml_diff>